<commit_message>
Cahier de recette : impression cadree sur la largeur d'une page A4 paysage
Mode d'emploi contenu dans les colonnes du tableau (cellules fusionnees, retour a la
ligne) : il ne deborde plus a droite. Zone d'impression A:N, toute la largeur sur une
page, marges reduites, centrage, en-tete du tableau repete, pied « Page n / N »,
largeurs de colonnes reparties. Verifie en PDF : 13 pages A4 paysage, 14 colonnes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NbgujfuPhMZiLjntCb4NUj
</commit_message>
<xml_diff>
--- a/docs/recette/Cahier_de_recette_Prestige.xlsx
+++ b/docs/recette/Cahier_de_recette_Prestige.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Cahier de recette" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Cahier de recette'!$A$1:$N$350</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Cahier de recette'!$12:$12</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Cahier de recette'!$A$12:$N$350</definedName>
   </definedNames>
@@ -3455,7 +3456,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3483,8 +3484,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -3857,25 +3858,37 @@
   <dimension ref="A1:N350"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="9"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -3895,7 +3908,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
         <v>5</v>
       </c>
@@ -3914,8 +3927,13 @@
       <c r="I5" s="8" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+    </row>
+    <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
@@ -3937,8 +3955,13 @@
       <c r="I6" s="8" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+    </row>
+    <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
         <v>11</v>
       </c>
@@ -3960,8 +3983,13 @@
       <c r="I7" s="8" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+    </row>
+    <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
         <v>14</v>
       </c>
@@ -3976,8 +4004,13 @@
       <c r="I8" s="8" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+    </row>
+    <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
         <v>16</v>
       </c>
@@ -3992,6 +4025,11 @@
       <c r="I9" s="8" t="s">
         <v>17</v>
       </c>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
@@ -4118,7 +4156,7 @@
       <c r="M14" s="11"/>
       <c r="N14" s="11"/>
     </row>
-    <row r="15" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="n">
         <v>3</v>
       </c>
@@ -4186,7 +4224,7 @@
       <c r="M16" s="11"/>
       <c r="N16" s="11"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="n">
         <v>5</v>
       </c>
@@ -4220,7 +4258,7 @@
       <c r="M17" s="11"/>
       <c r="N17" s="11"/>
     </row>
-    <row r="18" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="n">
         <v>6</v>
       </c>
@@ -4458,7 +4496,7 @@
       <c r="M24" s="11"/>
       <c r="N24" s="11"/>
     </row>
-    <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="n">
         <v>13</v>
       </c>
@@ -4492,7 +4530,7 @@
       <c r="M25" s="11"/>
       <c r="N25" s="11"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="n">
         <v>14</v>
       </c>
@@ -4594,7 +4632,7 @@
       <c r="M28" s="11"/>
       <c r="N28" s="11"/>
     </row>
-    <row r="29" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="n">
         <v>17</v>
       </c>
@@ -4798,7 +4836,7 @@
       <c r="M34" s="11"/>
       <c r="N34" s="11"/>
     </row>
-    <row r="35" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="n">
         <v>23</v>
       </c>
@@ -4934,7 +4972,7 @@
       <c r="M38" s="11"/>
       <c r="N38" s="11"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="n">
         <v>27</v>
       </c>
@@ -5036,7 +5074,7 @@
       <c r="M41" s="11"/>
       <c r="N41" s="11"/>
     </row>
-    <row r="42" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="13" t="n">
         <v>30</v>
       </c>
@@ -5104,7 +5142,7 @@
       <c r="M43" s="11"/>
       <c r="N43" s="11"/>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="13" t="n">
         <v>32</v>
       </c>
@@ -5138,7 +5176,7 @@
       <c r="M44" s="11"/>
       <c r="N44" s="11"/>
     </row>
-    <row r="45" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="10" t="n">
         <v>33</v>
       </c>
@@ -5308,7 +5346,7 @@
       <c r="M49" s="11"/>
       <c r="N49" s="11"/>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="13" t="n">
         <v>38</v>
       </c>
@@ -5342,7 +5380,7 @@
       <c r="M50" s="11"/>
       <c r="N50" s="11"/>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="10" t="n">
         <v>39</v>
       </c>
@@ -5376,7 +5414,7 @@
       <c r="M51" s="11"/>
       <c r="N51" s="11"/>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="13" t="n">
         <v>40</v>
       </c>
@@ -5410,7 +5448,7 @@
       <c r="M52" s="11"/>
       <c r="N52" s="11"/>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="10" t="n">
         <v>41</v>
       </c>
@@ -5444,7 +5482,7 @@
       <c r="M53" s="11"/>
       <c r="N53" s="11"/>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="13" t="n">
         <v>42</v>
       </c>
@@ -5546,7 +5584,7 @@
       <c r="M56" s="11"/>
       <c r="N56" s="11"/>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="10" t="n">
         <v>45</v>
       </c>
@@ -6158,7 +6196,7 @@
       <c r="M74" s="11"/>
       <c r="N74" s="11"/>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="10" t="n">
         <v>63</v>
       </c>
@@ -6260,7 +6298,7 @@
       <c r="M77" s="11"/>
       <c r="N77" s="11"/>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="13" t="n">
         <v>66</v>
       </c>
@@ -6294,7 +6332,7 @@
       <c r="M78" s="11"/>
       <c r="N78" s="11"/>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="10" t="n">
         <v>67</v>
       </c>
@@ -6328,7 +6366,7 @@
       <c r="M79" s="11"/>
       <c r="N79" s="11"/>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="13" t="n">
         <v>68</v>
       </c>
@@ -6362,7 +6400,7 @@
       <c r="M80" s="11"/>
       <c r="N80" s="11"/>
     </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="10" t="n">
         <v>69</v>
       </c>
@@ -6396,7 +6434,7 @@
       <c r="M81" s="11"/>
       <c r="N81" s="11"/>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="13" t="n">
         <v>70</v>
       </c>
@@ -6430,7 +6468,7 @@
       <c r="M82" s="11"/>
       <c r="N82" s="11"/>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="10" t="n">
         <v>71</v>
       </c>
@@ -6498,7 +6536,7 @@
       <c r="M84" s="11"/>
       <c r="N84" s="11"/>
     </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="10" t="n">
         <v>73</v>
       </c>
@@ -6668,7 +6706,7 @@
       <c r="M89" s="11"/>
       <c r="N89" s="11"/>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="13" t="n">
         <v>78</v>
       </c>
@@ -6736,7 +6774,7 @@
       <c r="M91" s="11"/>
       <c r="N91" s="11"/>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="13" t="n">
         <v>80</v>
       </c>
@@ -6838,7 +6876,7 @@
       <c r="M94" s="11"/>
       <c r="N94" s="11"/>
     </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="10" t="n">
         <v>83</v>
       </c>
@@ -6872,7 +6910,7 @@
       <c r="M95" s="11"/>
       <c r="N95" s="11"/>
     </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="13" t="n">
         <v>84</v>
       </c>
@@ -6940,7 +6978,7 @@
       <c r="M97" s="11"/>
       <c r="N97" s="11"/>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="13" t="n">
         <v>86</v>
       </c>
@@ -7008,7 +7046,7 @@
       <c r="M99" s="11"/>
       <c r="N99" s="11"/>
     </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="13" t="n">
         <v>88</v>
       </c>
@@ -7110,7 +7148,7 @@
       <c r="M102" s="11"/>
       <c r="N102" s="11"/>
     </row>
-    <row r="103" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="10" t="n">
         <v>91</v>
       </c>
@@ -7348,7 +7386,7 @@
       <c r="M109" s="11"/>
       <c r="N109" s="11"/>
     </row>
-    <row r="110" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="13" t="n">
         <v>98</v>
       </c>
@@ -7824,7 +7862,7 @@
       <c r="M123" s="11"/>
       <c r="N123" s="11"/>
     </row>
-    <row r="124" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="13" t="n">
         <v>112</v>
       </c>
@@ -7858,7 +7896,7 @@
       <c r="M124" s="11"/>
       <c r="N124" s="11"/>
     </row>
-    <row r="125" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="10" t="n">
         <v>113</v>
       </c>
@@ -7892,7 +7930,7 @@
       <c r="M125" s="11"/>
       <c r="N125" s="11"/>
     </row>
-    <row r="126" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="13" t="n">
         <v>114</v>
       </c>
@@ -7994,7 +8032,7 @@
       <c r="M128" s="11"/>
       <c r="N128" s="11"/>
     </row>
-    <row r="129" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="10" t="n">
         <v>117</v>
       </c>
@@ -8062,7 +8100,7 @@
       <c r="M130" s="11"/>
       <c r="N130" s="11"/>
     </row>
-    <row r="131" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="10" t="n">
         <v>119</v>
       </c>
@@ -8096,7 +8134,7 @@
       <c r="M131" s="11"/>
       <c r="N131" s="11"/>
     </row>
-    <row r="132" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="13" t="n">
         <v>120</v>
       </c>
@@ -8198,7 +8236,7 @@
       <c r="M134" s="11"/>
       <c r="N134" s="11"/>
     </row>
-    <row r="135" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="10" t="n">
         <v>123</v>
       </c>
@@ -8266,7 +8304,7 @@
       <c r="M136" s="11"/>
       <c r="N136" s="11"/>
     </row>
-    <row r="137" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="10" t="n">
         <v>125</v>
       </c>
@@ -8300,7 +8338,7 @@
       <c r="M137" s="11"/>
       <c r="N137" s="11"/>
     </row>
-    <row r="138" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="13" t="n">
         <v>126</v>
       </c>
@@ -8504,7 +8542,7 @@
       <c r="M143" s="11"/>
       <c r="N143" s="11"/>
     </row>
-    <row r="144" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="13" t="n">
         <v>132</v>
       </c>
@@ -8674,7 +8712,7 @@
       <c r="M148" s="11"/>
       <c r="N148" s="11"/>
     </row>
-    <row r="149" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="149" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="10" t="n">
         <v>137</v>
       </c>
@@ -8844,7 +8882,7 @@
       <c r="M153" s="11"/>
       <c r="N153" s="11"/>
     </row>
-    <row r="154" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="13" t="n">
         <v>142</v>
       </c>
@@ -8946,7 +8984,7 @@
       <c r="M156" s="11"/>
       <c r="N156" s="11"/>
     </row>
-    <row r="157" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="10" t="n">
         <v>145</v>
       </c>
@@ -9082,7 +9120,7 @@
       <c r="M160" s="11"/>
       <c r="N160" s="11"/>
     </row>
-    <row r="161" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="10" t="n">
         <v>149</v>
       </c>
@@ -9116,7 +9154,7 @@
       <c r="M161" s="11"/>
       <c r="N161" s="11"/>
     </row>
-    <row r="162" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="13" t="n">
         <v>150</v>
       </c>
@@ -9150,7 +9188,7 @@
       <c r="M162" s="11"/>
       <c r="N162" s="11"/>
     </row>
-    <row r="163" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="10" t="n">
         <v>151</v>
       </c>
@@ -9184,7 +9222,7 @@
       <c r="M163" s="11"/>
       <c r="N163" s="11"/>
     </row>
-    <row r="164" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="13" t="n">
         <v>152</v>
       </c>
@@ -9252,7 +9290,7 @@
       <c r="M165" s="11"/>
       <c r="N165" s="11"/>
     </row>
-    <row r="166" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="13" t="n">
         <v>154</v>
       </c>
@@ -9388,7 +9426,7 @@
       <c r="M169" s="11"/>
       <c r="N169" s="11"/>
     </row>
-    <row r="170" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="13" t="n">
         <v>158</v>
       </c>
@@ -9456,7 +9494,7 @@
       <c r="M171" s="11"/>
       <c r="N171" s="11"/>
     </row>
-    <row r="172" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="13" t="n">
         <v>160</v>
       </c>
@@ -9490,7 +9528,7 @@
       <c r="M172" s="11"/>
       <c r="N172" s="11"/>
     </row>
-    <row r="173" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="10" t="n">
         <v>161</v>
       </c>
@@ -9558,7 +9596,7 @@
       <c r="M174" s="11"/>
       <c r="N174" s="11"/>
     </row>
-    <row r="175" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="10" t="n">
         <v>163</v>
       </c>
@@ -9660,7 +9698,7 @@
       <c r="M177" s="11"/>
       <c r="N177" s="11"/>
     </row>
-    <row r="178" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="178" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="13" t="n">
         <v>166</v>
       </c>
@@ -9694,7 +9732,7 @@
       <c r="M178" s="11"/>
       <c r="N178" s="11"/>
     </row>
-    <row r="179" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="10" t="n">
         <v>167</v>
       </c>
@@ -9796,7 +9834,7 @@
       <c r="M181" s="11"/>
       <c r="N181" s="11"/>
     </row>
-    <row r="182" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="182" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="13" t="n">
         <v>170</v>
       </c>
@@ -9830,7 +9868,7 @@
       <c r="M182" s="11"/>
       <c r="N182" s="11"/>
     </row>
-    <row r="183" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="183" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="10" t="n">
         <v>171</v>
       </c>
@@ -10000,7 +10038,7 @@
       <c r="M187" s="11"/>
       <c r="N187" s="11"/>
     </row>
-    <row r="188" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="188" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="13" t="n">
         <v>176</v>
       </c>
@@ -10102,7 +10140,7 @@
       <c r="M190" s="11"/>
       <c r="N190" s="11"/>
     </row>
-    <row r="191" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="191" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="10" t="n">
         <v>179</v>
       </c>
@@ -10170,7 +10208,7 @@
       <c r="M192" s="11"/>
       <c r="N192" s="11"/>
     </row>
-    <row r="193" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="193" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="10" t="n">
         <v>181</v>
       </c>
@@ -10204,7 +10242,7 @@
       <c r="M193" s="11"/>
       <c r="N193" s="11"/>
     </row>
-    <row r="194" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="13" t="n">
         <v>182</v>
       </c>
@@ -10238,7 +10276,7 @@
       <c r="M194" s="11"/>
       <c r="N194" s="11"/>
     </row>
-    <row r="195" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="195" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="10" t="n">
         <v>183</v>
       </c>
@@ -10272,7 +10310,7 @@
       <c r="M195" s="11"/>
       <c r="N195" s="11"/>
     </row>
-    <row r="196" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="196" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="13" t="n">
         <v>184</v>
       </c>
@@ -10306,7 +10344,7 @@
       <c r="M196" s="11"/>
       <c r="N196" s="11"/>
     </row>
-    <row r="197" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="197" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="10" t="n">
         <v>185</v>
       </c>
@@ -10374,7 +10412,7 @@
       <c r="M198" s="11"/>
       <c r="N198" s="11"/>
     </row>
-    <row r="199" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="199" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="10" t="n">
         <v>187</v>
       </c>
@@ -10476,7 +10514,7 @@
       <c r="M201" s="11"/>
       <c r="N201" s="11"/>
     </row>
-    <row r="202" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="202" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="13" t="n">
         <v>190</v>
       </c>
@@ -10646,7 +10684,7 @@
       <c r="M206" s="11"/>
       <c r="N206" s="11"/>
     </row>
-    <row r="207" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="10" t="n">
         <v>195</v>
       </c>
@@ -10680,7 +10718,7 @@
       <c r="M207" s="11"/>
       <c r="N207" s="11"/>
     </row>
-    <row r="208" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="208" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="13" t="n">
         <v>196</v>
       </c>
@@ -10714,7 +10752,7 @@
       <c r="M208" s="11"/>
       <c r="N208" s="11"/>
     </row>
-    <row r="209" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="209" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="10" t="n">
         <v>197</v>
       </c>
@@ -10748,7 +10786,7 @@
       <c r="M209" s="11"/>
       <c r="N209" s="11"/>
     </row>
-    <row r="210" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="210" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="13" t="n">
         <v>198</v>
       </c>
@@ -10782,7 +10820,7 @@
       <c r="M210" s="11"/>
       <c r="N210" s="11"/>
     </row>
-    <row r="211" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="211" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="10" t="n">
         <v>199</v>
       </c>
@@ -10850,7 +10888,7 @@
       <c r="M212" s="11"/>
       <c r="N212" s="11"/>
     </row>
-    <row r="213" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="213" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="10" t="n">
         <v>201</v>
       </c>
@@ -10884,7 +10922,7 @@
       <c r="M213" s="11"/>
       <c r="N213" s="11"/>
     </row>
-    <row r="214" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="214" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="13" t="n">
         <v>202</v>
       </c>
@@ -10918,7 +10956,7 @@
       <c r="M214" s="11"/>
       <c r="N214" s="11"/>
     </row>
-    <row r="215" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="215" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="10" t="n">
         <v>203</v>
       </c>
@@ -11054,7 +11092,7 @@
       <c r="M218" s="11"/>
       <c r="N218" s="11"/>
     </row>
-    <row r="219" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="219" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="10" t="n">
         <v>207</v>
       </c>
@@ -11088,7 +11126,7 @@
       <c r="M219" s="11"/>
       <c r="N219" s="11"/>
     </row>
-    <row r="220" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="220" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="13" t="n">
         <v>208</v>
       </c>
@@ -11122,7 +11160,7 @@
       <c r="M220" s="11"/>
       <c r="N220" s="11"/>
     </row>
-    <row r="221" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="221" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="10" t="n">
         <v>209</v>
       </c>
@@ -11156,7 +11194,7 @@
       <c r="M221" s="11"/>
       <c r="N221" s="11"/>
     </row>
-    <row r="222" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="222" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="13" t="n">
         <v>210</v>
       </c>
@@ -11224,7 +11262,7 @@
       <c r="M223" s="11"/>
       <c r="N223" s="11"/>
     </row>
-    <row r="224" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="224" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="13" t="n">
         <v>212</v>
       </c>
@@ -11258,7 +11296,7 @@
       <c r="M224" s="11"/>
       <c r="N224" s="11"/>
     </row>
-    <row r="225" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="225" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="10" t="n">
         <v>213</v>
       </c>
@@ -11326,7 +11364,7 @@
       <c r="M226" s="11"/>
       <c r="N226" s="11"/>
     </row>
-    <row r="227" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="227" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="10" t="n">
         <v>215</v>
       </c>
@@ -11360,7 +11398,7 @@
       <c r="M227" s="11"/>
       <c r="N227" s="11"/>
     </row>
-    <row r="228" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="228" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="13" t="n">
         <v>216</v>
       </c>
@@ -11394,7 +11432,7 @@
       <c r="M228" s="11"/>
       <c r="N228" s="11"/>
     </row>
-    <row r="229" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="229" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="10" t="n">
         <v>217</v>
       </c>
@@ -11496,7 +11534,7 @@
       <c r="M231" s="11"/>
       <c r="N231" s="11"/>
     </row>
-    <row r="232" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="232" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="13" t="n">
         <v>220</v>
       </c>
@@ -11530,7 +11568,7 @@
       <c r="M232" s="11"/>
       <c r="N232" s="11"/>
     </row>
-    <row r="233" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="233" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="10" t="n">
         <v>221</v>
       </c>
@@ -11564,7 +11602,7 @@
       <c r="M233" s="11"/>
       <c r="N233" s="11"/>
     </row>
-    <row r="234" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="234" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="13" t="n">
         <v>222</v>
       </c>
@@ -11598,7 +11636,7 @@
       <c r="M234" s="11"/>
       <c r="N234" s="11"/>
     </row>
-    <row r="235" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="235" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="10" t="n">
         <v>223</v>
       </c>
@@ -11632,7 +11670,7 @@
       <c r="M235" s="11"/>
       <c r="N235" s="11"/>
     </row>
-    <row r="236" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="236" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="13" t="n">
         <v>224</v>
       </c>
@@ -11700,7 +11738,7 @@
       <c r="M237" s="11"/>
       <c r="N237" s="11"/>
     </row>
-    <row r="238" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="238" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="13" t="n">
         <v>226</v>
       </c>
@@ -11870,7 +11908,7 @@
       <c r="M242" s="11"/>
       <c r="N242" s="11"/>
     </row>
-    <row r="243" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="243" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="10" t="n">
         <v>231</v>
       </c>
@@ -11972,7 +12010,7 @@
       <c r="M245" s="11"/>
       <c r="N245" s="11"/>
     </row>
-    <row r="246" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="246" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="13" t="n">
         <v>234</v>
       </c>
@@ -12006,7 +12044,7 @@
       <c r="M246" s="11"/>
       <c r="N246" s="11"/>
     </row>
-    <row r="247" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="247" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="10" t="n">
         <v>235</v>
       </c>
@@ -12448,7 +12486,7 @@
       <c r="M259" s="11"/>
       <c r="N259" s="11"/>
     </row>
-    <row r="260" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="260" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="13" t="n">
         <v>248</v>
       </c>
@@ -12618,7 +12656,7 @@
       <c r="M264" s="11"/>
       <c r="N264" s="11"/>
     </row>
-    <row r="265" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="265" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A265" s="10" t="n">
         <v>253</v>
       </c>
@@ -12890,7 +12928,7 @@
       <c r="M272" s="11"/>
       <c r="N272" s="11"/>
     </row>
-    <row r="273" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="273" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="10" t="n">
         <v>261</v>
       </c>
@@ -12924,7 +12962,7 @@
       <c r="M273" s="11"/>
       <c r="N273" s="11"/>
     </row>
-    <row r="274" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="274" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A274" s="13" t="n">
         <v>262</v>
       </c>
@@ -12992,7 +13030,7 @@
       <c r="M275" s="11"/>
       <c r="N275" s="11"/>
     </row>
-    <row r="276" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="276" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="13" t="n">
         <v>264</v>
       </c>
@@ -13026,7 +13064,7 @@
       <c r="M276" s="11"/>
       <c r="N276" s="11"/>
     </row>
-    <row r="277" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="277" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="10" t="n">
         <v>265</v>
       </c>
@@ -13060,7 +13098,7 @@
       <c r="M277" s="11"/>
       <c r="N277" s="11"/>
     </row>
-    <row r="278" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="278" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A278" s="13" t="n">
         <v>266</v>
       </c>
@@ -13094,7 +13132,7 @@
       <c r="M278" s="11"/>
       <c r="N278" s="11"/>
     </row>
-    <row r="279" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="279" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A279" s="10" t="n">
         <v>267</v>
       </c>
@@ -13162,7 +13200,7 @@
       <c r="M280" s="11"/>
       <c r="N280" s="11"/>
     </row>
-    <row r="281" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="281" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A281" s="10" t="n">
         <v>269</v>
       </c>
@@ -13196,7 +13234,7 @@
       <c r="M281" s="11"/>
       <c r="N281" s="11"/>
     </row>
-    <row r="282" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="282" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A282" s="13" t="n">
         <v>270</v>
       </c>
@@ -13230,7 +13268,7 @@
       <c r="M282" s="11"/>
       <c r="N282" s="11"/>
     </row>
-    <row r="283" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="283" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="10" t="n">
         <v>271</v>
       </c>
@@ -13264,7 +13302,7 @@
       <c r="M283" s="11"/>
       <c r="N283" s="11"/>
     </row>
-    <row r="284" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="284" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="13" t="n">
         <v>272</v>
       </c>
@@ -13298,7 +13336,7 @@
       <c r="M284" s="11"/>
       <c r="N284" s="11"/>
     </row>
-    <row r="285" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="285" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="10" t="n">
         <v>273</v>
       </c>
@@ -13400,7 +13438,7 @@
       <c r="M287" s="11"/>
       <c r="N287" s="11"/>
     </row>
-    <row r="288" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="288" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A288" s="13" t="n">
         <v>276</v>
       </c>
@@ -13468,7 +13506,7 @@
       <c r="M289" s="11"/>
       <c r="N289" s="11"/>
     </row>
-    <row r="290" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="290" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A290" s="13" t="n">
         <v>278</v>
       </c>
@@ -13502,7 +13540,7 @@
       <c r="M290" s="11"/>
       <c r="N290" s="11"/>
     </row>
-    <row r="291" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="291" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A291" s="10" t="n">
         <v>279</v>
       </c>
@@ -13536,7 +13574,7 @@
       <c r="M291" s="11"/>
       <c r="N291" s="11"/>
     </row>
-    <row r="292" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="292" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A292" s="13" t="n">
         <v>280</v>
       </c>
@@ -13570,7 +13608,7 @@
       <c r="M292" s="11"/>
       <c r="N292" s="11"/>
     </row>
-    <row r="293" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="293" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A293" s="10" t="n">
         <v>281</v>
       </c>
@@ -13638,7 +13676,7 @@
       <c r="M294" s="11"/>
       <c r="N294" s="11"/>
     </row>
-    <row r="295" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="295" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A295" s="10" t="n">
         <v>283</v>
       </c>
@@ -13672,7 +13710,7 @@
       <c r="M295" s="11"/>
       <c r="N295" s="11"/>
     </row>
-    <row r="296" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="296" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A296" s="13" t="n">
         <v>284</v>
       </c>
@@ -13706,7 +13744,7 @@
       <c r="M296" s="11"/>
       <c r="N296" s="11"/>
     </row>
-    <row r="297" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="297" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A297" s="10" t="n">
         <v>285</v>
       </c>
@@ -13740,7 +13778,7 @@
       <c r="M297" s="11"/>
       <c r="N297" s="11"/>
     </row>
-    <row r="298" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="298" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A298" s="13" t="n">
         <v>286</v>
       </c>
@@ -13774,7 +13812,7 @@
       <c r="M298" s="11"/>
       <c r="N298" s="11"/>
     </row>
-    <row r="299" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="299" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A299" s="10" t="n">
         <v>287</v>
       </c>
@@ -13910,7 +13948,7 @@
       <c r="M302" s="11"/>
       <c r="N302" s="11"/>
     </row>
-    <row r="303" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="303" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A303" s="10" t="n">
         <v>291</v>
       </c>
@@ -13944,7 +13982,7 @@
       <c r="M303" s="11"/>
       <c r="N303" s="11"/>
     </row>
-    <row r="304" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="304" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A304" s="13" t="n">
         <v>292</v>
       </c>
@@ -13978,7 +14016,7 @@
       <c r="M304" s="11"/>
       <c r="N304" s="11"/>
     </row>
-    <row r="305" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="305" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A305" s="10" t="n">
         <v>293</v>
       </c>
@@ -14012,7 +14050,7 @@
       <c r="M305" s="11"/>
       <c r="N305" s="11"/>
     </row>
-    <row r="306" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="306" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A306" s="13" t="n">
         <v>294</v>
       </c>
@@ -14046,7 +14084,7 @@
       <c r="M306" s="11"/>
       <c r="N306" s="11"/>
     </row>
-    <row r="307" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="307" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A307" s="10" t="n">
         <v>295</v>
       </c>
@@ -14080,7 +14118,7 @@
       <c r="M307" s="11"/>
       <c r="N307" s="11"/>
     </row>
-    <row r="308" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="308" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A308" s="13" t="n">
         <v>296</v>
       </c>
@@ -14114,7 +14152,7 @@
       <c r="M308" s="11"/>
       <c r="N308" s="11"/>
     </row>
-    <row r="309" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="309" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A309" s="10" t="n">
         <v>297</v>
       </c>
@@ -14148,7 +14186,7 @@
       <c r="M309" s="11"/>
       <c r="N309" s="11"/>
     </row>
-    <row r="310" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="310" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A310" s="13" t="n">
         <v>298</v>
       </c>
@@ -14250,7 +14288,7 @@
       <c r="M312" s="11"/>
       <c r="N312" s="11"/>
     </row>
-    <row r="313" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="313" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A313" s="10" t="n">
         <v>301</v>
       </c>
@@ -14284,7 +14322,7 @@
       <c r="M313" s="11"/>
       <c r="N313" s="11"/>
     </row>
-    <row r="314" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="314" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A314" s="13" t="n">
         <v>302</v>
       </c>
@@ -14522,7 +14560,7 @@
       <c r="M320" s="11"/>
       <c r="N320" s="11"/>
     </row>
-    <row r="321" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="321" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A321" s="10" t="n">
         <v>309</v>
       </c>
@@ -14556,7 +14594,7 @@
       <c r="M321" s="11"/>
       <c r="N321" s="11"/>
     </row>
-    <row r="322" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="322" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A322" s="13" t="n">
         <v>310</v>
       </c>
@@ -14590,7 +14628,7 @@
       <c r="M322" s="11"/>
       <c r="N322" s="11"/>
     </row>
-    <row r="323" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="323" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A323" s="10" t="n">
         <v>311</v>
       </c>
@@ -14624,7 +14662,7 @@
       <c r="M323" s="11"/>
       <c r="N323" s="11"/>
     </row>
-    <row r="324" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="324" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A324" s="13" t="n">
         <v>312</v>
       </c>
@@ -14692,7 +14730,7 @@
       <c r="M325" s="11"/>
       <c r="N325" s="11"/>
     </row>
-    <row r="326" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="326" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A326" s="13" t="n">
         <v>314</v>
       </c>
@@ -15032,7 +15070,7 @@
       <c r="M335" s="11"/>
       <c r="N335" s="11"/>
     </row>
-    <row r="336" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="336" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A336" s="13" t="n">
         <v>324</v>
       </c>
@@ -15066,7 +15104,7 @@
       <c r="M336" s="11"/>
       <c r="N336" s="11"/>
     </row>
-    <row r="337" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="337" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A337" s="10" t="n">
         <v>325</v>
       </c>
@@ -15100,7 +15138,7 @@
       <c r="M337" s="11"/>
       <c r="N337" s="11"/>
     </row>
-    <row r="338" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="338" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A338" s="13" t="n">
         <v>326</v>
       </c>
@@ -15134,7 +15172,7 @@
       <c r="M338" s="11"/>
       <c r="N338" s="11"/>
     </row>
-    <row r="339" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="339" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A339" s="10" t="n">
         <v>327</v>
       </c>
@@ -15338,7 +15376,7 @@
       <c r="M344" s="11"/>
       <c r="N344" s="11"/>
     </row>
-    <row r="345" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="345" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A345" s="10" t="n">
         <v>333</v>
       </c>
@@ -15372,7 +15410,7 @@
       <c r="M345" s="11"/>
       <c r="N345" s="11"/>
     </row>
-    <row r="346" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="346" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A346" s="13" t="n">
         <v>334</v>
       </c>
@@ -15406,7 +15444,7 @@
       <c r="M346" s="11"/>
       <c r="N346" s="11"/>
     </row>
-    <row r="347" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="347" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A347" s="10" t="n">
         <v>335</v>
       </c>
@@ -15508,7 +15546,7 @@
       <c r="M349" s="11"/>
       <c r="N349" s="11"/>
     </row>
-    <row r="350" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="350" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A350" s="13" t="n">
         <v>338</v>
       </c>
@@ -15544,6 +15582,14 @@
     </row>
   </sheetData>
   <autoFilter ref="A12:N350"/>
+  <mergeCells count="6">
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="I5:N5"/>
+    <mergeCell ref="I6:N6"/>
+    <mergeCell ref="I7:N7"/>
+    <mergeCell ref="I8:N8"/>
+    <mergeCell ref="I9:N9"/>
+  </mergeCells>
   <conditionalFormatting sqref="L13:L350">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"OK"</formula>
@@ -15565,12 +15611,12 @@
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.2" right="0.2" top="0.35" bottom="0.35" header="0.511811023622047" footer="0.15"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;8 Page &amp;P / &amp;N&amp;R&amp;8 Cahier de recette Prestige</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>